<commit_message>
Re-export spreadsheet; mulligan UI and bag draw count tweaks
- Remove Ambidextrous aura from spreadsheet export; bat_wing point_value 1

- Show mulligan button and counter throughout the brew scene

- Bag count drops by 1 as each hand-draw fly animation starts
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Alchemy Roguelite Godot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12E4A11-680E-477D-BC8F-4F5198EC1A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2462F335-DF5C-41E1-833C-F4080A6FB6B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="146">
   <si>
     <t>id</t>
   </si>
@@ -428,15 +428,6 @@
   </si>
   <si>
     <t>Threshold increased by 50% and gold gained is double</t>
-  </si>
-  <si>
-    <t>ambidextrous</t>
-  </si>
-  <si>
-    <t>Ambidextrous</t>
-  </si>
-  <si>
-    <t>Ingredients are added to the cauldron 2 at a time</t>
   </si>
   <si>
     <t>in_rhythm</t>
@@ -1461,7 +1452,7 @@
         <v>63</v>
       </c>
       <c r="E18" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18">
         <v>0</v>
@@ -1864,7 +1855,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2137,10 +2128,10 @@
         <v>145</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="E12" s="4">
         <v>0</v>
@@ -2152,32 +2143,9 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E13" s="4">
-        <v>0</v>
-      </c>
-      <c r="F13" s="4">
-        <v>100</v>
-      </c>
-      <c r="G13" s="4">
-        <v>100</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="D2:D200" xr:uid="{00000000-0002-0000-0300-000000000000}">
+    <dataValidation type="list" sqref="D2:D199" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"normal,boss"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Clamp boss threshold to minimum of 1
- Add MIN_BOSS_THRESHOLD and clamp after penalties, discounts, and aura modifiers

- Re-export ingredients spreadsheet
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Alchemy Roguelite Godot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE0719F-4F31-461A-98B9-1A0E6F087886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E49DA1-9571-4358-80F0-0D267D7C5301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1596,7 +1596,7 @@
         <v>75</v>
       </c>
       <c r="E22" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" s="9">
         <v>0</v>

</xml_diff>

<commit_message>
Re-export spreadsheet and fix voodoo/bat wing interaction
- Mandrake boss threshold discount back to 1; leech 3% reduction and 1 point

- Defer voodoo doll copy until bat wing picker selection resolves

- Re-export ingredients.xlsx to JSON
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Alchemy Roguelite Godot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3E49DA1-9571-4358-80F0-0D267D7C5301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4905FF08-4B67-4D5A-94D9-30D5B55514BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -178,9 +178,6 @@
     <t>Mandrake</t>
   </si>
   <si>
-    <t>The next boss has -2 score threshold</t>
-  </si>
-  <si>
     <t>dragon_fruit</t>
   </si>
   <si>
@@ -250,9 +247,6 @@
     <t>Leech</t>
   </si>
   <si>
-    <t>10% of your score this round is applied to the next boss instead</t>
-  </si>
-  <si>
     <t>thorns</t>
   </si>
   <si>
@@ -470,6 +464,12 @@
   </si>
   <si>
     <t>Regular Boss</t>
+  </si>
+  <si>
+    <t>3% of your score this round is applied to the next boss instead</t>
+  </si>
+  <si>
+    <t>The next boss has -1 score threshold</t>
   </si>
 </sst>
 </file>
@@ -921,27 +921,27 @@
   <sheetData>
     <row r="1" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
@@ -949,37 +949,37 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -1361,7 +1361,7 @@
         <v>50</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>51</v>
+        <v>148</v>
       </c>
       <c r="E14" s="4">
         <v>3</v>
@@ -1381,16 +1381,16 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B15" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="11" t="s">
         <v>53</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>54</v>
       </c>
       <c r="E15" s="4">
         <v>10</v>
@@ -1410,16 +1410,16 @@
     </row>
     <row r="16" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B16" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>57</v>
       </c>
       <c r="E16" s="4">
         <v>1</v>
@@ -1439,16 +1439,16 @@
     </row>
     <row r="17" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B17" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" s="9" t="s">
+      <c r="D17" s="11" t="s">
         <v>59</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>60</v>
       </c>
       <c r="E17" s="9">
         <v>4</v>
@@ -1468,16 +1468,16 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B18" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="9" t="s">
+      <c r="D18" s="11" t="s">
         <v>62</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>63</v>
       </c>
       <c r="E18" s="9">
         <v>1</v>
@@ -1497,16 +1497,16 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B19" t="s">
-        <v>64</v>
-      </c>
-      <c r="C19" s="9" t="s">
+      <c r="D19" s="11" t="s">
         <v>65</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>66</v>
       </c>
       <c r="E19" s="9">
         <v>1</v>
@@ -1526,16 +1526,16 @@
     </row>
     <row r="20" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C20" s="9" t="s">
+      <c r="D20" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="E20" s="9">
         <v>1</v>
@@ -1555,16 +1555,16 @@
     </row>
     <row r="21" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B21" t="s">
-        <v>70</v>
-      </c>
-      <c r="C21" s="9" t="s">
+      <c r="D21" s="11" t="s">
         <v>71</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>72</v>
       </c>
       <c r="E21" s="9">
         <v>4</v>
@@ -1584,16 +1584,16 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B22" t="s">
+        <v>72</v>
+      </c>
+      <c r="C22" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="B22" t="s">
-        <v>73</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>74</v>
-      </c>
       <c r="D22" s="11" t="s">
-        <v>75</v>
+        <v>147</v>
       </c>
       <c r="E22" s="9">
         <v>1</v>
@@ -1613,16 +1613,16 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>76</v>
-      </c>
-      <c r="B23" t="s">
-        <v>76</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>78</v>
       </c>
       <c r="E23" s="9">
         <v>1</v>
@@ -1642,16 +1642,16 @@
     </row>
     <row r="24" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B24" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D24" s="11" t="s">
         <v>79</v>
-      </c>
-      <c r="B24" t="s">
-        <v>79</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>81</v>
       </c>
       <c r="E24" s="9">
         <v>2</v>
@@ -1671,13 +1671,13 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>82</v>
-      </c>
-      <c r="C25" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>84</v>
       </c>
       <c r="E25" s="9">
         <v>1</v>
@@ -1697,13 +1697,13 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>85</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>87</v>
       </c>
       <c r="E26" s="9">
         <v>2</v>
@@ -1723,13 +1723,13 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D27" s="11" t="s">
         <v>88</v>
-      </c>
-      <c r="C27" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>90</v>
       </c>
       <c r="E27" s="9">
         <v>3</v>
@@ -1749,16 +1749,16 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>91</v>
-      </c>
-      <c r="B28" t="s">
-        <v>91</v>
-      </c>
-      <c r="C28" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>93</v>
       </c>
       <c r="E28" s="9">
         <v>3</v>
@@ -1778,16 +1778,16 @@
     </row>
     <row r="29" spans="1:9" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B29" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>94</v>
-      </c>
-      <c r="B29" t="s">
-        <v>94</v>
-      </c>
-      <c r="C29" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>96</v>
       </c>
       <c r="E29" s="9">
         <v>2</v>
@@ -1830,10 +1830,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1854,7 +1854,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B4" s="4">
         <v>2</v>
@@ -1906,30 +1906,30 @@
         <v>3</v>
       </c>
       <c r="D1" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="G1" s="7" t="s">
         <v>112</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="D2" s="8" t="s">
         <v>116</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>118</v>
       </c>
       <c r="E2" s="8">
         <v>1</v>
@@ -1943,16 +1943,16 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>121</v>
-      </c>
       <c r="D3" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E3" s="8">
         <v>0</v>
@@ -1966,16 +1966,16 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="D4" s="8" t="s">
         <v>123</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>125</v>
       </c>
       <c r="E4" s="8">
         <v>-1</v>
@@ -1989,16 +1989,16 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>128</v>
-      </c>
       <c r="D5" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E5" s="8">
         <v>-2</v>
@@ -2012,16 +2012,16 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>131</v>
-      </c>
       <c r="D6" s="8" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E6" s="8">
         <v>0</v>
@@ -2035,16 +2035,16 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>134</v>
-      </c>
       <c r="D7" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E7" s="4">
         <v>0</v>
@@ -2058,16 +2058,16 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>137</v>
-      </c>
       <c r="D8" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E8" s="4">
         <v>0</v>
@@ -2081,16 +2081,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>140</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E9" s="4">
         <v>0</v>
@@ -2104,16 +2104,16 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>143</v>
-      </c>
       <c r="D10" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E10" s="4">
         <v>0</v>
@@ -2127,16 +2127,16 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>146</v>
-      </c>
       <c r="D11" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E11" s="4">
         <v>0</v>
@@ -2150,16 +2150,16 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E12" s="4">
         <v>0</v>

</xml_diff>

<commit_message>
Add hand-brew ingredients and fix fairy poof, severed hands, mulligan, fish bones art
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Auras" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -36,16 +36,6 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="FF444444"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="FF0000FF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -94,6 +84,16 @@
       <color rgb="FF444444"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -130,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -142,18 +142,27 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -533,28 +542,28 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>1. Edit the Ingredients, Auras, and StarterBag sheets.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>2. Save this file.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>3. Run: py tools/export_ingredients.py</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>4. Play the game in Godot (it loads data/*.json).</t>
         </is>
@@ -564,49 +573,49 @@
       <c r="A7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Ingredients: id, art, display_name, description, point_value, explosive_value, shop_cost, rarity, shop_available</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Auras: id, display_name, description, pool, explosion_limit_modifier, score_multiplier_percent, gold_multiplier_percent</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>pool = normal (regular levels) or boss (every 5th level). Multipliers use 100 = no change.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>art = PNG filename in assets/cards/ingredients/ (blank uses id).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>shop_available FALSE = starter-only, never appears in the shop.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Description: effect text (normal) or flavor text (italicize in Excel).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Example art file: assets/cards/ingredients/boom_berry.png</t>
         </is>
@@ -623,18 +632,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="61.77734375" customWidth="1" style="11" min="4" max="4"/>
+    <col width="61.77734375" customWidth="1" style="9" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="11.109375" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -653,7 +663,7 @@
           <t>display_name</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="8" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -700,7 +710,7 @@
           <t>Small Boom Berry</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t>An unassuming, delicious fruit!</t>
         </is>
@@ -739,7 +749,7 @@
           <t>Boom Berry</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>An unassuming, delicious fruit!</t>
         </is>
@@ -778,7 +788,7 @@
           <t>Large Boom Berry</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>An unassuming, delicious fruit!</t>
         </is>
@@ -807,12 +817,17 @@
           <t>pumpkin</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>pumpkin</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Pumpkin</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Pumpkin!</t>
         </is>
@@ -841,12 +856,17 @@
           <t>jackolantern</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>jackolantern</t>
+        </is>
+      </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Jack-O-Lantern</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Also a Pumpkin</t>
         </is>
@@ -875,12 +895,17 @@
           <t>chili_pepper</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>chili_pepper</t>
+        </is>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Chili Pepper</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>Spicy!</t>
         </is>
@@ -892,7 +917,7 @@
         <v>2</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
@@ -909,12 +934,17 @@
           <t>red_mushroom</t>
         </is>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>red_mushroom</t>
+        </is>
+      </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Red Mushroom</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Has +1 for each pumpkin in your cauldron (Maximum of +3)</t>
         </is>
@@ -943,12 +973,17 @@
           <t>lightning_in_a_bottle</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>lightning_in_a_bottle</t>
+        </is>
+      </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Lightning in a Bottle</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Play 3 random ingredients from your cauldron</t>
         </is>
@@ -977,12 +1012,17 @@
           <t>eyeball</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>eyeball</t>
+        </is>
+      </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Eyeball</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Look at the next 3 ingredients you will draw</t>
         </is>
@@ -994,7 +1034,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
@@ -1011,12 +1051,17 @@
           <t>unicorn_horn</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>unicorn_horn</t>
+        </is>
+      </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Unicorn Horn</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Your next ingredients explosiveness is cured if it has any</t>
         </is>
@@ -1024,7 +1069,7 @@
       <c r="E11" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="7" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="4" t="n">
@@ -1038,6 +1083,11 @@
       <c r="I11" s="4" t="b">
         <v>1</v>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>shadow ban</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1045,12 +1095,17 @@
           <t>parrot</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>parrot</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Par-rot</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>your next ingredient is added twice</t>
         </is>
@@ -1079,12 +1134,17 @@
           <t>feather</t>
         </is>
       </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>feather</t>
+        </is>
+      </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Feather</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>Gain 1 Gold</t>
         </is>
@@ -1096,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
@@ -1113,12 +1173,17 @@
           <t>mandrake</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>mandrake</t>
+        </is>
+      </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Mandrake</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>The next boss has -1 score threshold</t>
         </is>
@@ -1130,7 +1195,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
@@ -1157,7 +1222,7 @@
           <t>Dragon's Fruit</t>
         </is>
       </c>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Dragon's find them delicious!</t>
         </is>
@@ -1169,7 +1234,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
@@ -1196,7 +1261,7 @@
           <t>Pheonix Feather</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>If this would cause your cauldron to explode, instead, set explosiveness to 0 and reshuffle all ingredients back into your bag (you keep your score)</t>
         </is>
@@ -1220,7 +1285,7 @@
       </c>
     </row>
     <row r="17" ht="28.8" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>gloom_weed</t>
         </is>
@@ -1230,36 +1295,36 @@
           <t>gloom_weed</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Gloom Weed</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>If this is your last ingredient added to the cauldron when you stop brewing, double your gold gained</t>
         </is>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="9" t="n">
+      <c r="F17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I17" s="9" t="b">
+      <c r="I17" s="7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>bat_wing</t>
         </is>
@@ -1269,445 +1334,1089 @@
           <t>bat_wing</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>Bat Wing</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Draw 3 ingredients from your bag and select 1 to add to your cauldron</t>
         </is>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="9" t="n">
+      <c r="G18" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="H18" s="9" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I18" s="9" t="b">
+      <c r="I18" s="7" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>rat</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>rat</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Rat</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>Has +1 score for each rat added in a row (Max +4)</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" ht="28.8" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>voodoo_doll</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>voodoo_doll</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Voodoo Doll</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Becomes a permanent copy of the next ingredient you add to your cauldron</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" ht="28.8" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>frog_leg</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>frog_leg</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Frog Leg</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>If you would expload this jumps out of your cauldron instead (You won't be quick enough to catch it)</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>leech</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>leech</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Leech</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>3% of your score this round is applied to the next boss instead</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I22" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>thorns</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>thorns</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Thorns</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Add the current explosiveness to the score</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" ht="28.8" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>garlic</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>garlic</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Garlic</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>increase explosiveness threshold by 1. If you've added Garlic already, this does nothing</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="I24" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>newt_tail</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>newt_tail</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Newt Tail</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Adds +1 score for each explosive ingredient you add after this</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>cinnamon</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>cinnamon</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Cinnamon</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>If you end on an even number score gain 2 gold</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F26" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>sage</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Sage</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Adds 1 free reroll to the shop</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>eye_of_ender</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>eye_of_ender</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>Eye of Ender</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Gain 1 Mulligan this round</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" ht="28.8" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>lucky_coin</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>lucky_coin</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Lucky Coin</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>If you don't swap this hand, gain 1 extra swap next hand, If you do, gain +2 gold</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>holy_grail</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>holy_grail</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Holy Grail</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Increase explosion limit by 1</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F30" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>ice_cube</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ice_cube</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Ice Cube</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>For the next 4 ingredients, explosiveness is added normally unless that ingredient would make the cauldron explode</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>shrunken_head</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>shrunken_head</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>Shrunken Head</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Your next hand is only 4 ingredients</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="I32" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>jar_of_dirt</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>jar_of_dirt</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Jar of Dirt</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>Add a pumpkin to your bag</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>stirring_spoon</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>stirring_spoon</t>
+        </is>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Stirring Spoon</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Your next hand has an additional swap</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H34" s="7" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="I34" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>fish_bones</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>fish_bones</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Fish Bones</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>Reduce your cauldron's score by 1 and gain 2 gold</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>fairy_in_a_cage</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>fairy_in_a_cage</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Fairy in a Cage</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Your next ingredient disappears forever</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>shadow ban</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28.8" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>booberry</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>booberry</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Boo-berry</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>End of hand: lose 2 explosiveness</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>chicken</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>chicken</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Chicken</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>This cannot make your cauldron explode</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>spider</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>spider</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C39" s="7" t="inlineStr">
         <is>
           <t>Spider</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>Has +1 score for each spider added in a row (Max +4)</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="9" t="n">
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="9" t="inlineStr">
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I19" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" ht="28.8" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
-        <is>
-          <t>voodoo_doll</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>voodoo_doll</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Voodoo Doll</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>Becomes a permanent copy of the next ingredient you add to your cauldron</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="9" t="n">
+      <c r="I39" s="7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>poison_apple</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>poison_apple</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Poison Apple</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>In 2 hands, gain 3 explosiveness</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>cobbler</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>cobbler</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Cobbler</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>Adjacent Boomberries are +2 explosiveness and +10 score</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F41" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I20" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" ht="28.8" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
-        <is>
-          <t>frog_leg</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>frog_leg</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>Frog Leg</t>
-        </is>
-      </c>
-      <c r="D21" s="11" t="inlineStr">
-        <is>
-          <t>If you would expload this jumps out of your cauldron instead (You won't be quick enough to catch it)</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="n">
+      <c r="I41" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>growth_potion</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>growth_potion</t>
+        </is>
+      </c>
+      <c r="C42" s="7" t="inlineStr">
+        <is>
+          <t>Growth Potion</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>The next 4 ingredients stats are doubled</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>severed_right_hand</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>severed_right_hand</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Severed Right Hand</t>
+        </is>
+      </c>
+      <c r="D43" s="9" t="inlineStr">
+        <is>
+          <t>Gains 1 score for each ingredient to the left</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>severed_left_hand</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>severed_left_hand</t>
+        </is>
+      </c>
+      <c r="C44" s="7" t="inlineStr">
+        <is>
+          <t>Severed Left Hand</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Gains 1 score for each ingredient to the right</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>11</v>
+      </c>
+      <c r="H44" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>juggling_club</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>juggling_club</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Juggling Club</t>
+        </is>
+      </c>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>Your next 3 hands have an additional swap</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F21" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>legendary</t>
-        </is>
-      </c>
-      <c r="I21" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>leech</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>leech</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Leech</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>3% of your score this round is applied to the next boss instead</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
+      <c r="F45" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I22" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>thorns</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>thorns</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Thorns</t>
-        </is>
-      </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>Add the current explosiveness to the score</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="H23" s="9" t="inlineStr">
-        <is>
-          <t>uncommon</t>
-        </is>
-      </c>
-      <c r="I23" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" ht="28.8" customHeight="1">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>garlic</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>garlic</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Garlic</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>increase explosiveness threshold by 1. If you've added Garlic already, this does nothing</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="H24" s="9" t="inlineStr">
-        <is>
-          <t>epic</t>
-        </is>
-      </c>
-      <c r="I24" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>newt_tail</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Newt Tail</t>
-        </is>
-      </c>
-      <c r="D25" s="11" t="inlineStr">
-        <is>
-          <t>Adds +1 score for each explosive ingredient you add after this</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="H25" s="9" t="inlineStr">
-        <is>
-          <t>rare</t>
-        </is>
-      </c>
-      <c r="I25" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>cinnamon</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Cinnamon</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>If you end on an even number score gain 2 gold</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="H26" s="9" t="inlineStr">
-        <is>
-          <t>uncommon</t>
-        </is>
-      </c>
-      <c r="I26" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>sage</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Sage</t>
-        </is>
-      </c>
-      <c r="D27" s="11" t="inlineStr">
-        <is>
-          <t>Adds 1 free reroll to the shop</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="H27" s="9" t="inlineStr">
-        <is>
-          <t>uncommon</t>
-        </is>
-      </c>
-      <c r="I27" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>eye_of_ender</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>eye_of_ender</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Eye of Ender</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>Gain 1 Mulligan this round</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="H28" s="9" t="inlineStr">
-        <is>
-          <t>epic</t>
-        </is>
-      </c>
-      <c r="I28" s="9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" ht="28.8" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>lucky_coin</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>lucky_coin</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Lucky Coin</t>
-        </is>
-      </c>
-      <c r="D29" s="11" t="inlineStr">
-        <is>
-          <t>If you don't swap this hand, gain +2 gold, If you do, gain 1 extra swap next hand</t>
-        </is>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="F29" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="H29" s="9" t="inlineStr">
-        <is>
-          <t>rare</t>
-        </is>
-      </c>
-      <c r="I29" s="9" t="b">
+      <c r="I45" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1773,7 +2482,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>spider</t>
+          <t>rat</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -1811,402 +2520,440 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="72.44140625" customWidth="1" min="3" max="3"/>
+    <col width="58.21875" customWidth="1" style="15" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="27.6640625" customWidth="1" min="5" max="5"/>
-    <col width="26.44140625" customWidth="1" min="6" max="6"/>
-    <col width="25.77734375" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>pool</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>pool_unlock_level</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>explosion_limit_modifier</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>score_multiplier_percent</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>gold_multiplier_percent</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>stable_brew</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>Stable Brew</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="14" t="inlineStr">
         <is>
           <t>Explosion limit +1 this level.</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E2" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="8" t="n">
+      <c r="E2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="H2" s="12" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>gold_rush</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Gold Rush</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>Gold earned +25% this level.</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E3" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="8" t="n">
+      <c r="E3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="H3" s="12" t="n">
         <v>125</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>shaky_hands</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Shaky Hands</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>Explosion limit -1 this level.</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" s="12" t="n">
         <v>-1</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="G4" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="H4" s="12" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>volatile_brew</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Volatile Brew</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Explosion limit -2.</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="F5" s="12" t="n">
         <v>-2</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="G5" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="H5" s="12" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>stingy</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Stingy</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Gold earned -25%.</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E6" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="8" t="n">
+      <c r="E6" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="H6" s="12" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>low_expectations</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Low Expectations</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>Threshold reduced by 15%</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="4" t="n">
+      <c r="E7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="12" t="n">
         <v>85</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="12" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>under_pressure</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Under Pressure</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Increase threshold and gold gain by 15%</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="4" t="n">
+      <c r="E8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="12" t="n">
         <v>115</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="12" t="n">
         <v>115</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="9" ht="28.2" customHeight="1">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>in_rhythm</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>In Rhythm</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>every 3rd ingredient added to the cauldron has double score and explosiveness</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4" t="n">
+      <c r="E9" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="12" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>practice brew</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Practice Brew</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>You may restart the brew at anypoint before it explodes</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="4" t="n">
+      <c r="E10" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="12" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>regular_brew</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Regular Brew</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Nothing special</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="4" t="n">
+      <c r="E11" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="12" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>regular_boss</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Regular Boss</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Nothing special</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="4" t="n">
+      <c r="E12" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="12" t="n">
         <v>100</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D199" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"normal,boss"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync ingredient, aura, and starter bag data from spreadsheet
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Alchemy Roguelite Godot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4209954-1AAD-48FD-B587-0CA73F151C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F312DEA-8D19-4C0A-9A34-BA120FF681D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="202">
   <si>
     <t>id</t>
   </si>
@@ -620,6 +620,15 @@
   </si>
   <si>
     <t>Regular Boss</t>
+  </si>
+  <si>
+    <t>Bubbling Brew</t>
+  </si>
+  <si>
+    <t>bubbling_brew</t>
+  </si>
+  <si>
+    <t>every 3rd ingredient added to the cauldron jumps back into your bag.</t>
   </si>
 </sst>
 </file>
@@ -2552,7 +2561,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2875,6 +2884,32 @@
         <v>100</v>
       </c>
     </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="E13" s="4">
+        <v>1</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+      <c r="G13" s="4">
+        <v>100</v>
+      </c>
+      <c r="H13" s="4">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" sqref="D2:D200" xr:uid="{00000000-0002-0000-0300-000000000000}">

</xml_diff>

<commit_message>
Add Honey ingredient: skip left neighbor on hand play
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" state="visible" r:id="rId1"/>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -2431,6 +2431,40 @@
         </is>
       </c>
       <c r="I45" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>honey</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Honey</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>The ingredient to the left</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>12</v>
+      </c>
+      <c r="H46" s="7" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="I46" s="7" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3012,12 +3046,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20.77734375" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="59.6640625" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3048,7 +3082,7 @@
           <t>Pumpkin Necklace</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Pumpkins gain +1 score for each pumpkin played before it in a row</t>
         </is>
@@ -3065,28 +3099,444 @@
           <t>Red Mushroom Trinket</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Red mushrooms can score a maximum of 6 instead of 4</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>rat_trinket</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Rat Trinket</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Rats can score a maximum of 6 instead of 4</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>jar_of_flies</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Jar of Flies</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Batwing has an option to reroll choices once</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>pocket_watch</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Pocket Watch</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Every 21st ingredient added has double stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>time_turner</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Time Turner</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Click to redraw your hand and lose this trinket</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>jar_of_froglegs</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Jar of Froglegs</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Your froglegs jump back into your bag at the end of the level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>voodoo_doll_trinket</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Voodoo Doll</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Voodoo Dolls become common in the shop and cost 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>pristine_feather</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Pristine Feather</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Your feathers are played twice</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>beating_heart</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Beating Heart</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Gain a life and add a 3 Boomberry to your bag</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>gecko_feet</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Gecko Feet</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Every 11 ingredients stays in your hand</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n"/>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n"/>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n"/>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n"/>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n"/>
+      <c r="B22" s="4" t="n"/>
+      <c r="C22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n"/>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n"/>
+      <c r="B24" s="4" t="n"/>
+      <c r="C24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n"/>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n"/>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="n"/>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n"/>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n"/>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n"/>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n"/>
+      <c r="B32" s="4" t="n"/>
+      <c r="C32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n"/>
+      <c r="B33" s="4" t="n"/>
+      <c r="C33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n"/>
+      <c r="B34" s="4" t="n"/>
+      <c r="C34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n"/>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n"/>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n"/>
+      <c r="B38" s="4" t="n"/>
+      <c r="C38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n"/>
+      <c r="B39" s="4" t="n"/>
+      <c r="C39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n"/>
+      <c r="B40" s="4" t="n"/>
+      <c r="C40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n"/>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n"/>
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n"/>
+      <c r="B43" s="4" t="n"/>
+      <c r="C43" s="4" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n"/>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n"/>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n"/>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n"/>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n"/>
+      <c r="B48" s="4" t="n"/>
+      <c r="C48" s="4" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n"/>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="4" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n"/>
+      <c r="B50" s="4" t="n"/>
+      <c r="C50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n"/>
+      <c r="B51" s="4" t="n"/>
+      <c r="C51" s="4" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n"/>
+      <c r="B52" s="4" t="n"/>
+      <c r="C52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n"/>
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n"/>
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n"/>
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="4" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n"/>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n"/>
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n"/>
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n"/>
+      <c r="B59" s="4" t="n"/>
+      <c r="C59" s="4" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n"/>
+      <c r="B60" s="4" t="n"/>
+      <c r="C60" s="4" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n"/>
+      <c r="B61" s="4" t="n"/>
+      <c r="C61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n"/>
+      <c r="B62" s="4" t="n"/>
+      <c r="C62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n"/>
+      <c r="B63" s="4" t="n"/>
+      <c r="C63" s="4" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n"/>
+      <c r="B64" s="4" t="n"/>
+      <c r="C64" s="4" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n"/>
+      <c r="B65" s="4" t="n"/>
+      <c r="C65" s="4" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n"/>
+      <c r="B66" s="4" t="n"/>
+      <c r="C66" s="4" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n"/>
+      <c r="B67" s="4" t="n"/>
+      <c r="C67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n"/>
+      <c r="B68" s="4" t="n"/>
+      <c r="C68" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add trinkets, bat wing slot resolve, and spreadsheet sync
Implement Voodoo Doll, Pristine Feather, Time Turner, Jar of Froglegs, and Jar of Dirt with art and verification scripts. Bat wing picker choices resolve in the source hand slot with hand-aware Cobbler logic. Sync ingredients.xlsx from JSON and update shop generation for Voodoo Doll trinket pricing and rarity.
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -100,8 +100,16 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +136,11 @@
         <fgColor rgb="FFE8E8E8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -141,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,6 +190,10 @@
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -646,1533 +663,1522 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J46"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:I46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="61.77734375" customWidth="1" style="9" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="11.109375" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>art</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="D1" s="8" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>point_value</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>explosive_value</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>shop_cost</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>rarity</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="17" t="inlineStr">
         <is>
           <t>shop_available</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>boom_berry_1</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>boom_berry</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Small Boom Berry</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>An unassuming, delicious fruit!</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="E2" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I2" s="6" t="b">
+      <c r="I2" s="18" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>boom_berry_2</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>boom_berry</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>Boom Berry</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>An unassuming, delicious fruit!</t>
         </is>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F3" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="G3" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I3" s="6" t="b">
+      <c r="I3" s="18" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>boom_berry_3</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>boom_berry</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Large Boom Berry</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>An unassuming, delicious fruit!</t>
         </is>
       </c>
-      <c r="E4" s="6" t="n">
+      <c r="E4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="F4" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="G4" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I4" s="6" t="b">
+      <c r="I4" s="18" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>pumpkin</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>pumpkin</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Pumpkin</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Pumpkin!</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="4" t="n">
+      <c r="E5" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I5" s="4" t="b">
+      <c r="I5" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>jackolantern</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>jackolantern</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Jack-O-Lantern</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Also a Pumpkin</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="F6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4" t="n">
+      <c r="F6" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I6" s="4" t="b">
+      <c r="I6" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>chili_pepper</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>chili_pepper</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Chili Pepper</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Spicy!</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F7" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="G7" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I7" s="4" t="b">
+      <c r="I7" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>red_mushroom</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>red_mushroom</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Red Mushroom</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Has +1 for each pumpkin in your cauldron (Maximum of +3)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="4" t="n">
+      <c r="E8" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I8" s="4" t="b">
+      <c r="I8" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>lightning_in_a_bottle</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>lightning_in_a_bottle</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Lightning in a Bottle</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Play 3 random ingredients from your cauldron</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4" t="n">
+      <c r="F9" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I9" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" ht="28.8" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="I9" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>eyeball</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>eyeball</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>Eyeball</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Look at the next 3 ingredients you will draw</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="4" t="n">
+      <c r="E10" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I10" s="4" t="b">
+      <c r="I10" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>unicorn_horn</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>unicorn_horn</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Unicorn Horn</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Your next ingredients explosiveness is cured if it has any</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="4" t="n">
+      <c r="F11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="18" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I11" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>shadow ban</t>
-        </is>
+      <c r="I11" s="18" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>parrot</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>parrot</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Par-rot</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>your next ingredient is added twice</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="4" t="n">
+      <c r="E12" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="18" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I12" s="4" t="b">
+      <c r="I12" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>feather</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>feather</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Feather</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Gain 1 Gold</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4" t="n">
+      <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I13" s="4" t="b">
+      <c r="I13" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>mandrake</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>mandrake</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr">
         <is>
           <t>Mandrake</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>The next boss has -1 score threshold</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="4" t="n">
+      <c r="F14" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I14" s="4" t="b">
+      <c r="I14" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>dragon_fruit</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>dragon_fruit</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Dragon's Fruit</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Dragon's find them delicious!</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="F15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="4" t="n">
+      <c r="F15" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I15" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" ht="28.8" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="I15" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
         <is>
           <t>pheonix_feather</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>pheonix_feather</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="18" t="inlineStr">
         <is>
           <t>Pheonix Feather</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>If this would cause your cauldron to explode, instead, set explosiveness to 0 and reshuffle all ingredients back into your bag (you keep your score)</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" t="n">
+      <c r="E16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H16" s="18" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I16" s="4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" ht="28.8" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="I16" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>gloom_weed</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>gloom_weed</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Gloom Weed</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>If this is your last ingredient added to the cauldron when you stop brewing, double your gold gained</t>
         </is>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="7" t="n">
+      <c r="F17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I17" s="7" t="b">
+      <c r="I17" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>bat_wing</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>bat_wing</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr">
         <is>
           <t>Bat Wing</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Draw 3 ingredients from your bag and select 1 to add to your cauldron</t>
         </is>
       </c>
-      <c r="E18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="7" t="n">
+      <c r="E18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="H18" s="7" t="inlineStr">
+      <c r="H18" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I18" s="7" t="b">
+      <c r="I18" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>rat</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>rat</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr">
         <is>
           <t>Rat</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Has +1 score for each rat added in a row (Max +4)</t>
         </is>
       </c>
-      <c r="E19" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="7" t="n">
+      <c r="E19" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I19" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" ht="28.8" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="I19" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>voodoo_doll</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="18" t="inlineStr">
         <is>
           <t>voodoo_doll</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr">
         <is>
           <t>Voodoo Doll</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Becomes a permanent copy of the next ingredient you add to your cauldron</t>
         </is>
       </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="7" t="n">
+      <c r="E20" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I20" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" ht="28.8" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="I20" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
         <is>
           <t>frog_leg</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>frog_leg</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="18" t="inlineStr">
         <is>
           <t>Frog Leg</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>If you would expload this jumps out of your cauldron instead (You won't be quick enough to catch it)</t>
         </is>
       </c>
-      <c r="E21" s="7" t="n">
+      <c r="E21" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F21" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="7" t="n">
+      <c r="F21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H21" s="18" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I21" s="7" t="b">
+      <c r="I21" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+      <c r="A22" s="18" t="inlineStr">
         <is>
           <t>leech</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>leech</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="18" t="inlineStr">
         <is>
           <t>Leech</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>3% of your score this round is applied to the next boss instead</t>
         </is>
       </c>
-      <c r="E22" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="7" t="n">
+      <c r="E22" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="H22" s="7" t="inlineStr">
+      <c r="H22" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I22" s="7" t="b">
+      <c r="I22" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>thorns</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>thorns</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="18" t="inlineStr">
         <is>
           <t>Thorns</t>
         </is>
       </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Add the current explosiveness to the score</t>
         </is>
       </c>
-      <c r="E23" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="7" t="n">
+      <c r="E23" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H23" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I23" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" ht="28.8" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="I23" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
         <is>
           <t>garlic</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>garlic</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C24" s="18" t="inlineStr">
         <is>
           <t>Garlic</t>
         </is>
       </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>increase explosiveness threshold by 1. If you've added Garlic already, this does nothing</t>
         </is>
       </c>
-      <c r="E24" s="7" t="n">
+      <c r="E24" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F24" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="7" t="n">
+      <c r="F24" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="H24" s="7" t="inlineStr">
+      <c r="H24" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I24" s="7" t="b">
+      <c r="I24" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>newt_tail</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>newt_tail</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Newt Tail</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Adds +1 score for each explosive ingredient you add after this</t>
         </is>
       </c>
-      <c r="E25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="7" t="n">
+      <c r="E25" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H25" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I25" s="7" t="b">
+      <c r="I25" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="18" t="inlineStr">
         <is>
           <t>cinnamon</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>cinnamon</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C26" s="18" t="inlineStr">
         <is>
           <t>Cinnamon</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>If you end on an even number score gain 2 gold</t>
         </is>
       </c>
-      <c r="E26" s="7" t="n">
+      <c r="E26" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F26" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="7" t="n">
+      <c r="F26" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H26" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I26" s="7" t="b">
+      <c r="I26" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="18" t="inlineStr">
         <is>
           <t>sage</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>sage</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>Sage</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Adds 1 free reroll to the shop</t>
         </is>
       </c>
-      <c r="E27" s="7" t="n">
+      <c r="E27" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="7" t="n">
+      <c r="F27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H27" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I27" s="7" t="b">
+      <c r="I27" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>eye_of_ender</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>eye_of_ender</t>
         </is>
       </c>
-      <c r="C28" s="7" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>Eye of Ender</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Gain 1 Mulligan this round</t>
         </is>
       </c>
-      <c r="E28" s="7" t="n">
+      <c r="E28" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F28" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="7" t="n">
+      <c r="F28" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="H28" s="7" t="inlineStr">
+      <c r="H28" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I28" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" ht="28.8" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="I28" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>lucky_coin</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>lucky_coin</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="18" t="inlineStr">
         <is>
           <t>Lucky Coin</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>If you don't swap this hand, gain 1 extra swap next hand, If you do, gain +2 gold</t>
         </is>
       </c>
-      <c r="E29" s="7" t="n">
+      <c r="E29" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F29" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="7" t="n">
+      <c r="F29" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="18" t="n">
         <v>13</v>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I29" s="7" t="b">
+      <c r="I29" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>holy_grail</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>holy_grail</t>
         </is>
       </c>
-      <c r="C30" s="7" t="inlineStr">
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Holy Grail</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Increase explosion limit by 1</t>
         </is>
       </c>
-      <c r="E30" s="7" t="n">
+      <c r="E30" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="7" t="n">
+      <c r="F30" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H30" s="18" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I30" s="7" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" ht="28.8" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="I30" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>ice_cube</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>ice_cube</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="18" t="inlineStr">
         <is>
           <t>Ice Cube</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>For the next 4 ingredients, explosiveness is added normally unless that ingredient would make the cauldron explode</t>
         </is>
       </c>
-      <c r="E31" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="7" t="n">
+      <c r="E31" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I31" s="7" t="b">
+      <c r="I31" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="7" t="inlineStr">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>shrunken_head</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>shrunken_head</t>
         </is>
       </c>
-      <c r="C32" s="7" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>Shrunken Head</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Your next hand is only 4 ingredients</t>
         </is>
       </c>
-      <c r="E32" s="7" t="n">
+      <c r="E32" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F32" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="7" t="n">
+      <c r="F32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="H32" s="7" t="inlineStr">
+      <c r="H32" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I32" s="7" t="b">
+      <c r="I32" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="18" t="inlineStr">
         <is>
           <t>jar_of_dirt</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>jar_of_dirt</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="18" t="inlineStr">
         <is>
           <t>Jar of Dirt</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Add a pumpkin to your bag</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="n">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Add a pumpkin to your bag. Breaks after 5 pumpkins.</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="7" t="n">
+      <c r="F33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H33" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I33" s="7" t="b">
+      <c r="I33" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>stirring_spoon</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>stirring_spoon</t>
         </is>
       </c>
-      <c r="C34" s="7" t="inlineStr">
+      <c r="C34" s="18" t="inlineStr">
         <is>
           <t>Stirring Spoon</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Your next hand has an additional swap</t>
         </is>
       </c>
-      <c r="E34" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="7" t="n">
+      <c r="E34" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H34" s="7" t="inlineStr">
+      <c r="H34" s="18" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I34" s="7" t="b">
+      <c r="I34" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>fish_bones</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="18" t="inlineStr">
         <is>
           <t>fish_bones</t>
         </is>
       </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="18" t="inlineStr">
         <is>
           <t>Fish Bones</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Reduce your cauldron's score by 1 and gain 2 gold</t>
         </is>
       </c>
-      <c r="E35" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="7" t="n">
+      <c r="E35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H35" s="7" t="inlineStr">
+      <c r="H35" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I35" s="7" t="b">
+      <c r="I35" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>fairy_in_a_cage</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="18" t="inlineStr">
         <is>
           <t>fairy_in_a_cage</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C36" s="18" t="inlineStr">
         <is>
           <t>Fairy in a Cage</t>
         </is>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Your next ingredient disappears forever</t>
         </is>
       </c>
-      <c r="E36" s="7" t="n">
+      <c r="E36" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="F36" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="7" t="n">
+      <c r="F36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="18" t="n">
         <v>50</v>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H36" s="18" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I36" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>shadow ban</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="28.8" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="I36" s="18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="inlineStr">
         <is>
           <t>booberry</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="18" t="inlineStr">
         <is>
           <t>booberry</t>
         </is>
       </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="18" t="inlineStr">
         <is>
           <t>Boo-berry</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>End of hand: lose 2 explosiveness</t>
         </is>
       </c>
-      <c r="E37" s="7" t="n">
+      <c r="E37" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F37" s="7" t="n">
+      <c r="F37" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="7" t="n">
+      <c r="G37" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H37" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I37" s="7" t="b">
+      <c r="I37" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>chicken</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="18" t="inlineStr">
         <is>
           <t>chicken</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
+      <c r="C38" s="18" t="inlineStr">
         <is>
           <t>Chicken</t>
         </is>
       </c>
-      <c r="D38" s="9" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>This cannot make your cauldron explode</t>
         </is>
       </c>
-      <c r="E38" s="7" t="n">
+      <c r="E38" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F38" s="7" t="n">
+      <c r="F38" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G38" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="G38" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I38" s="7" t="b">
+      <c r="I38" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+      <c r="A39" s="18" t="inlineStr">
         <is>
           <t>spider</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="18" t="inlineStr">
         <is>
           <t>spider</t>
         </is>
       </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="18" t="inlineStr">
         <is>
           <t>Spider</t>
         </is>
@@ -2182,289 +2188,294 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="E39" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="7" t="n">
+      <c r="E39" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="H39" s="7" t="inlineStr">
+      <c r="H39" s="18" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I39" s="7" t="b">
+      <c r="I39" s="18" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
+      <c r="A40" s="18" t="inlineStr">
         <is>
           <t>poison_apple</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="18" t="inlineStr">
         <is>
           <t>poison_apple</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C40" s="18" t="inlineStr">
         <is>
           <t>Poison Apple</t>
         </is>
       </c>
-      <c r="D40" s="9" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>In 2 hands, gain 3 explosiveness</t>
         </is>
       </c>
-      <c r="E40" s="7" t="n">
+      <c r="E40" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="F40" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="7" t="n">
+      <c r="F40" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="H40" s="7" t="inlineStr">
+      <c r="H40" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I40" s="7" t="b">
+      <c r="I40" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="18" t="inlineStr">
         <is>
           <t>cobbler</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="18" t="inlineStr">
         <is>
           <t>cobbler</t>
         </is>
       </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="18" t="inlineStr">
         <is>
           <t>Cobbler</t>
         </is>
       </c>
-      <c r="D41" s="9" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Adjacent Boomberries are +2 explosiveness and +10 score</t>
         </is>
       </c>
-      <c r="E41" s="7" t="n">
+      <c r="E41" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="7" t="n">
+      <c r="F41" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="H41" s="7" t="inlineStr">
+      <c r="H41" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I41" s="7" t="b">
+      <c r="I41" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>growth_potion</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="18" t="inlineStr">
         <is>
           <t>growth_potion</t>
         </is>
       </c>
-      <c r="C42" s="7" t="inlineStr">
+      <c r="C42" s="18" t="inlineStr">
         <is>
           <t>Growth Potion</t>
         </is>
       </c>
-      <c r="D42" s="9" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>The next 4 ingredients stats are doubled</t>
         </is>
       </c>
-      <c r="E42" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="7" t="n">
+      <c r="E42" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="H42" s="7" t="inlineStr">
+      <c r="H42" s="18" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I42" s="7" t="b">
+      <c r="I42" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A43" s="18" t="inlineStr">
         <is>
           <t>severed_right_hand</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="18" t="inlineStr">
         <is>
           <t>severed_right_hand</t>
         </is>
       </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="18" t="inlineStr">
         <is>
           <t>Severed Right Hand</t>
         </is>
       </c>
-      <c r="D43" s="9" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>Gains 1 score for each ingredient to the left</t>
         </is>
       </c>
-      <c r="E43" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="7" t="n">
+      <c r="E43" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="H43" s="7" t="inlineStr">
+      <c r="H43" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I43" s="7" t="b">
+      <c r="I43" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="A44" s="18" t="inlineStr">
         <is>
           <t>severed_left_hand</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="18" t="inlineStr">
         <is>
           <t>severed_left_hand</t>
         </is>
       </c>
-      <c r="C44" s="7" t="inlineStr">
+      <c r="C44" s="18" t="inlineStr">
         <is>
           <t>Severed Left Hand</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>Gains 1 score for each ingredient to the right</t>
         </is>
       </c>
-      <c r="E44" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="7" t="n">
+      <c r="E44" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="H44" s="7" t="inlineStr">
+      <c r="H44" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I44" s="7" t="b">
+      <c r="I44" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+      <c r="A45" s="18" t="inlineStr">
         <is>
           <t>juggling_club</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="18" t="inlineStr">
         <is>
           <t>juggling_club</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="18" t="inlineStr">
         <is>
           <t>Juggling Club</t>
         </is>
       </c>
-      <c r="D45" s="9" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Your next 3 hands have an additional swap</t>
         </is>
       </c>
-      <c r="E45" s="7" t="n">
+      <c r="E45" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="F45" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="7" t="n">
+      <c r="F45" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H45" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I45" s="7" t="b">
+      <c r="I45" s="18" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+      <c r="A46" s="18" t="inlineStr">
         <is>
           <t>honey</t>
         </is>
       </c>
-      <c r="C46" s="7" t="inlineStr">
+      <c r="B46" s="18" t="inlineStr">
+        <is>
+          <t>honey</t>
+        </is>
+      </c>
+      <c r="C46" s="18" t="inlineStr">
         <is>
           <t>Honey</t>
         </is>
       </c>
-      <c r="D46" s="9" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>The ingredient to the left</t>
         </is>
       </c>
-      <c r="E46" s="7" t="n">
+      <c r="E46" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F46" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="7" t="n">
+      <c r="F46" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="H46" s="7" t="inlineStr">
+      <c r="H46" s="18" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I46" s="7" t="b">
+      <c r="I46" s="18" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2478,7 +2489,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -2489,71 +2499,71 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>ingredient_id</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>boom_berry_1</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="18" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>pumpkin</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="18" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>rat</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="18" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>red_mushroom</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="18" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>boom_berry_2</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="18" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2569,463 +2579,465 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="58.21875" customWidth="1" style="15" min="3" max="3"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="8"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="17" t="inlineStr">
         <is>
           <t>pool</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="17" t="inlineStr">
         <is>
           <t>pool_unlock_level</t>
         </is>
       </c>
-      <c r="F1" s="11" t="inlineStr">
+      <c r="F1" s="17" t="inlineStr">
         <is>
           <t>explosion_limit_modifier</t>
         </is>
       </c>
-      <c r="G1" s="11" t="inlineStr">
+      <c r="G1" s="17" t="inlineStr">
         <is>
           <t>score_multiplier_percent</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="H1" s="17" t="inlineStr">
         <is>
           <t>gold_multiplier_percent</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>stable_brew</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Stable Brew</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="18" t="inlineStr">
         <is>
           <t>Explosion limit +1 this level.</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="18" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E2" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="12" t="n">
+      <c r="E2" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H2" s="12" t="n">
+      <c r="H2" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>gold_rush</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Gold Rush</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>Gold earned +25% this level.</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E3" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="12" t="n">
+      <c r="E3" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="18" t="n">
         <v>125</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>shaky_hands</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Shaky Hands</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Explosion limit -1 this level.</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="12" t="n">
+      <c r="F4" s="18" t="n">
         <v>-1</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>volatile_brew</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Volatile Brew</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Explosion limit -2.</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="18" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="18" t="n">
         <v>-2</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>stingy</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Stingy</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="18" t="inlineStr">
         <is>
           <t>Gold earned -25%.</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E6" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="12" t="n">
+      <c r="E6" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="18" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>low_expectations</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Low Expectations</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Threshold reduced by 15%</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E7" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="12" t="n">
+      <c r="E7" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="18" t="n">
         <v>85</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>under_pressure</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Under Pressure</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Increase threshold and gold gain by 15%</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="12" t="n">
+      <c r="E8" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="18" t="n">
         <v>115</v>
       </c>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="18" t="n">
         <v>115</v>
       </c>
     </row>
-    <row r="9" ht="28.2" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>in_rhythm</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>In Rhythm</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>every 3rd ingredient added to the cauldron has double score and explosiveness</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="12" t="n">
+      <c r="E9" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>practice brew</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Practice Brew</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="18" t="inlineStr">
         <is>
           <t>You may restart the brew at anypoint before it explodes</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E10" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="12" t="n">
+      <c r="E10" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H10" s="12" t="n">
+      <c r="H10" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>regular_brew</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Regular Brew</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Nothing special</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="18" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="12" t="n">
+      <c r="E11" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="H11" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>regular_boss</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Regular Boss</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr">
         <is>
           <t>Nothing special</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="18" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E12" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="12" t="n">
+      <c r="E12" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H12" s="12" t="n">
+      <c r="H12" s="18" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="13" ht="28.2" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>bubbling_brew</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>Bubbling Brew</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>every 3rd ingredient added to the cauldron jumps back into your bag.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="18" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="4" t="n">
+      <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" s="18" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3036,7 +3048,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -3046,497 +3057,217 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20.77734375" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="59.6640625" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="17" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="C1" s="16" t="inlineStr">
+      <c r="C1" s="17" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="18" t="inlineStr">
         <is>
           <t>pumpkin_trinket</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>Pumpkin Necklace</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Pumpkins gain +1 score for each pumpkin played before it in a row</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>red_mushroom_trinket</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Red Mushroom Trinket</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Red mushrooms can score a maximum of 6 instead of 4</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>rat_trinket</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Rat Trinket</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Rats can score a maximum of 6 instead of 4</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>jar_of_flies</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Jar of Flies</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Batwing has an option to reroll choices once</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>pocket_watch</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Pocket Watch</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Every 21st ingredient added has double stats</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>time_turner</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Time Turner</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Click to redraw your hand and lose this trinket</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>jar_of_froglegs</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Jar of Froglegs</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Your froglegs jump back into your bag at the end of the level.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>voodoo_doll_trinket</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Voodoo Doll</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Voodoo Dolls become common in the shop and cost 6</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>pristine_feather</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>Pristine Feather</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Your feathers are played twice</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>beating_heart</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Beating Heart</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Gain a life and add a 3 Boomberry to your bag</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>gecko_feet</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Gecko Feet</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Every 11 ingredients stays in your hand</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n"/>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
-      <c r="C15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n"/>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n"/>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
-      <c r="C19" s="4" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n"/>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="n"/>
-      <c r="C21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n"/>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="n"/>
-      <c r="C23" s="4" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n"/>
-      <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n"/>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="n"/>
-      <c r="C27" s="4" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n"/>
-      <c r="B28" s="4" t="n"/>
-      <c r="C28" s="4" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n"/>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n"/>
-      <c r="B30" s="4" t="n"/>
-      <c r="C30" s="4" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
-      <c r="C31" s="4" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n"/>
-      <c r="B32" s="4" t="n"/>
-      <c r="C32" s="4" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n"/>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
-      <c r="C35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n"/>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
-      <c r="C37" s="4" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n"/>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n"/>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n"/>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n"/>
-      <c r="B41" s="4" t="n"/>
-      <c r="C41" s="4" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n"/>
-      <c r="B42" s="4" t="n"/>
-      <c r="C42" s="4" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n"/>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n"/>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n"/>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n"/>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n"/>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n"/>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="n"/>
-      <c r="B51" s="4" t="n"/>
-      <c r="C51" s="4" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="n"/>
-      <c r="B52" s="4" t="n"/>
-      <c r="C52" s="4" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="4" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="n"/>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="n"/>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="n"/>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="n"/>
-      <c r="B57" s="4" t="n"/>
-      <c r="C57" s="4" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="n"/>
-      <c r="B58" s="4" t="n"/>
-      <c r="C58" s="4" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="n"/>
-      <c r="B59" s="4" t="n"/>
-      <c r="C59" s="4" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="n"/>
-      <c r="B60" s="4" t="n"/>
-      <c r="C60" s="4" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="n"/>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="4" t="n"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="n"/>
-      <c r="B62" s="4" t="n"/>
-      <c r="C62" s="4" t="n"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="n"/>
-      <c r="B63" s="4" t="n"/>
-      <c r="C63" s="4" t="n"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="n"/>
-      <c r="B64" s="4" t="n"/>
-      <c r="C64" s="4" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="4" t="n"/>
-      <c r="B65" s="4" t="n"/>
-      <c r="C65" s="4" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="n"/>
-      <c r="B66" s="4" t="n"/>
-      <c r="C66" s="4" t="n"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="n"/>
-      <c r="B67" s="4" t="n"/>
-      <c r="C67" s="4" t="n"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="n"/>
-      <c r="B68" s="4" t="n"/>
-      <c r="C68" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Expand Pristine Feather to all feather ingredients and sync spreadsheet
Match ingredient ids containing feather (including pheonix_feather) for double-play and hand icons. Sync ingredients.xlsx from runtime JSON data.
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,42 +41,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="FF0000FF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
@@ -98,38 +63,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
     </font>
     <font>
       <name val="Arial"/>
       <color rgb="000000FF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8E8E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8E8E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8E8E8"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -154,46 +99,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -573,28 +492,28 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>1. Edit the Ingredients, Auras, and StarterBag sheets.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>2. Save this file.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>3. Run: py tools/export_ingredients.py</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>4. Play the game in Godot (it loads data/*.json).</t>
         </is>
@@ -604,49 +523,49 @@
       <c r="A7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Ingredients: id, art, display_name, description, point_value, explosive_value, shop_cost, rarity, shop_available</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Auras: id, display_name, description, pool, explosion_limit_modifier, score_multiplier_percent, gold_multiplier_percent</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>pool = normal (regular levels) or boss (every 5th level). Multipliers use 100 = no change.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>art = PNG filename in assets/cards/ingredients/ (blank uses id).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>shop_available FALSE = starter-only, never appears in the shop.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Description: effect text (normal) or flavor text (italicize in Excel).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Example art file: assets/cards/ingredients/boom_berry.png</t>
         </is>
@@ -678,64 +597,64 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>art</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="D1" s="17" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="17" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>point_value</t>
         </is>
       </c>
-      <c r="F1" s="17" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>explosive_value</t>
         </is>
       </c>
-      <c r="G1" s="17" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>shop_cost</t>
         </is>
       </c>
-      <c r="H1" s="17" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>rarity</t>
         </is>
       </c>
-      <c r="I1" s="17" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>shop_available</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>boom_berry_1</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>boom_berry</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Small Boom Berry</t>
         </is>
@@ -745,36 +664,36 @@
           <t>An unassuming, delicious fruit!</t>
         </is>
       </c>
-      <c r="E2" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="18" t="inlineStr">
+      <c r="E2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I2" s="18" t="b">
+      <c r="I2" s="8" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>boom_berry_2</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>boom_berry</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Boom Berry</t>
         </is>
@@ -784,36 +703,36 @@
           <t>An unassuming, delicious fruit!</t>
         </is>
       </c>
-      <c r="E3" s="18" t="n">
+      <c r="E3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="18" t="inlineStr">
+      <c r="G3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I3" s="18" t="b">
+      <c r="I3" s="8" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>boom_berry_3</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>boom_berry</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Large Boom Berry</t>
         </is>
@@ -823,36 +742,36 @@
           <t>An unassuming, delicious fruit!</t>
         </is>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="G4" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I4" s="18" t="b">
+      <c r="I4" s="8" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>pumpkin</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>pumpkin</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Pumpkin</t>
         </is>
@@ -862,36 +781,36 @@
           <t>Pumpkin!</t>
         </is>
       </c>
-      <c r="E5" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="18" t="n">
+      <c r="E5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="18" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I5" s="18" t="b">
+      <c r="I5" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>jackolantern</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>jackolantern</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Jack-O-Lantern</t>
         </is>
@@ -901,36 +820,36 @@
           <t>Also a Pumpkin</t>
         </is>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F6" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="18" t="n">
+      <c r="F6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="8" t="n">
         <v>22</v>
       </c>
-      <c r="H6" s="18" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I6" s="18" t="b">
+      <c r="I6" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>chili_pepper</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>chili_pepper</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Chili Pepper</t>
         </is>
@@ -940,36 +859,36 @@
           <t>Spicy!</t>
         </is>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I7" s="18" t="b">
+      <c r="I7" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>red_mushroom</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>red_mushroom</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Red Mushroom</t>
         </is>
@@ -979,36 +898,36 @@
           <t>Has +1 for each pumpkin in your cauldron (Maximum of +3)</t>
         </is>
       </c>
-      <c r="E8" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="18" t="n">
+      <c r="E8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I8" s="18" t="b">
+      <c r="I8" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>lightning_in_a_bottle</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>lightning_in_a_bottle</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Lightning in a Bottle</t>
         </is>
@@ -1018,36 +937,36 @@
           <t>Play 3 random ingredients from your cauldron</t>
         </is>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="18" t="n">
+      <c r="F9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I9" s="18" t="b">
+      <c r="I9" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>eyeball</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>eyeball</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Eyeball</t>
         </is>
@@ -1057,36 +976,36 @@
           <t>Look at the next 3 ingredients you will draw</t>
         </is>
       </c>
-      <c r="E10" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="18" t="n">
+      <c r="E10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I10" s="18" t="b">
+      <c r="I10" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>unicorn_horn</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>unicorn_horn</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Unicorn Horn</t>
         </is>
@@ -1096,36 +1015,36 @@
           <t>Your next ingredients explosiveness is cured if it has any</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="18" t="n">
+      <c r="F11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="H11" s="18" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I11" s="18" t="b">
+      <c r="I11" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>parrot</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>parrot</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Par-rot</t>
         </is>
@@ -1135,36 +1054,36 @@
           <t>your next ingredient is added twice</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="18" t="n">
+      <c r="E12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="H12" s="18" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I12" s="18" t="b">
+      <c r="I12" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>feather</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>feather</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Feather</t>
         </is>
@@ -1174,36 +1093,36 @@
           <t>Gain 1 Gold</t>
         </is>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="18" t="n">
+      <c r="E13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I13" s="18" t="b">
+      <c r="I13" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>mandrake</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>mandrake</t>
         </is>
       </c>
-      <c r="C14" s="18" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Mandrake</t>
         </is>
@@ -1213,36 +1132,36 @@
           <t>The next boss has -1 score threshold</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="18" t="n">
+      <c r="F14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="H14" s="18" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I14" s="18" t="b">
+      <c r="I14" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>dragon_fruit</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>dragon_fruit</t>
         </is>
       </c>
-      <c r="C15" s="18" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>Dragon's Fruit</t>
         </is>
@@ -1252,36 +1171,36 @@
           <t>Dragon's find them delicious!</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="F15" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="18" t="n">
+      <c r="F15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I15" s="18" t="b">
+      <c r="I15" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>pheonix_feather</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>pheonix_feather</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>Pheonix Feather</t>
         </is>
@@ -1291,36 +1210,36 @@
           <t>If this would cause your cauldron to explode, instead, set explosiveness to 0 and reshuffle all ingredients back into your bag (you keep your score)</t>
         </is>
       </c>
-      <c r="E16" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G16" s="18" t="n">
+      <c r="E16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="H16" s="18" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I16" s="18" t="b">
+      <c r="I16" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>gloom_weed</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>gloom_weed</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>Gloom Weed</t>
         </is>
@@ -1330,36 +1249,36 @@
           <t>If this is your last ingredient added to the cauldron when you stop brewing, double your gold gained</t>
         </is>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E17" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="18" t="n">
+      <c r="F17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="H17" s="18" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I17" s="18" t="b">
+      <c r="I17" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>bat_wing</t>
         </is>
       </c>
-      <c r="B18" s="18" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>bat_wing</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Bat Wing</t>
         </is>
@@ -1369,36 +1288,36 @@
           <t>Draw 3 ingredients from your bag and select 1 to add to your cauldron</t>
         </is>
       </c>
-      <c r="E18" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="18" t="n">
+      <c r="E18" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="H18" s="18" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I18" s="18" t="b">
+      <c r="I18" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>rat</t>
         </is>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>rat</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Rat</t>
         </is>
@@ -1408,36 +1327,36 @@
           <t>Has +1 score for each rat added in a row (Max +4)</t>
         </is>
       </c>
-      <c r="E19" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="18" t="n">
+      <c r="E19" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="18" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I19" s="18" t="b">
+      <c r="I19" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>voodoo_doll</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>voodoo_doll</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Voodoo Doll</t>
         </is>
@@ -1447,36 +1366,36 @@
           <t>Becomes a permanent copy of the next ingredient you add to your cauldron</t>
         </is>
       </c>
-      <c r="E20" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="18" t="n">
+      <c r="E20" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="H20" s="18" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I20" s="18" t="b">
+      <c r="I20" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>frog_leg</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>frog_leg</t>
         </is>
       </c>
-      <c r="C21" s="18" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Frog Leg</t>
         </is>
@@ -1486,36 +1405,36 @@
           <t>If you would expload this jumps out of your cauldron instead (You won't be quick enough to catch it)</t>
         </is>
       </c>
-      <c r="E21" s="18" t="n">
+      <c r="E21" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F21" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="18" t="n">
+      <c r="F21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="H21" s="18" t="inlineStr">
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I21" s="18" t="b">
+      <c r="I21" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>leech</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>leech</t>
         </is>
       </c>
-      <c r="C22" s="18" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Leech</t>
         </is>
@@ -1525,36 +1444,36 @@
           <t>3% of your score this round is applied to the next boss instead</t>
         </is>
       </c>
-      <c r="E22" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="18" t="n">
+      <c r="E22" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="H22" s="18" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I22" s="18" t="b">
+      <c r="I22" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>thorns</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>thorns</t>
         </is>
       </c>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Thorns</t>
         </is>
@@ -1564,36 +1483,36 @@
           <t>Add the current explosiveness to the score</t>
         </is>
       </c>
-      <c r="E23" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="18" t="n">
+      <c r="E23" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="H23" s="18" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I23" s="18" t="b">
+      <c r="I23" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>garlic</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>garlic</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Garlic</t>
         </is>
@@ -1603,36 +1522,36 @@
           <t>increase explosiveness threshold by 1. If you've added Garlic already, this does nothing</t>
         </is>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="E24" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F24" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="18" t="n">
+      <c r="F24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="H24" s="18" t="inlineStr">
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I24" s="18" t="b">
+      <c r="I24" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>newt_tail</t>
         </is>
       </c>
-      <c r="B25" s="18" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>newt_tail</t>
         </is>
       </c>
-      <c r="C25" s="18" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Newt Tail</t>
         </is>
@@ -1642,36 +1561,36 @@
           <t>Adds +1 score for each explosive ingredient you add after this</t>
         </is>
       </c>
-      <c r="E25" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="18" t="n">
+      <c r="E25" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="H25" s="18" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I25" s="18" t="b">
+      <c r="I25" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>cinnamon</t>
         </is>
       </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>cinnamon</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Cinnamon</t>
         </is>
@@ -1681,36 +1600,36 @@
           <t>If you end on an even number score gain 2 gold</t>
         </is>
       </c>
-      <c r="E26" s="18" t="n">
+      <c r="E26" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F26" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="18" t="n">
+      <c r="F26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="H26" s="18" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I26" s="18" t="b">
+      <c r="I26" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>sage</t>
         </is>
       </c>
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>sage</t>
         </is>
       </c>
-      <c r="C27" s="18" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Sage</t>
         </is>
@@ -1720,36 +1639,36 @@
           <t>Adds 1 free reroll to the shop</t>
         </is>
       </c>
-      <c r="E27" s="18" t="n">
+      <c r="E27" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="18" t="n">
+      <c r="F27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="8" t="n">
         <v>16</v>
       </c>
-      <c r="H27" s="18" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I27" s="18" t="b">
+      <c r="I27" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>eye_of_ender</t>
         </is>
       </c>
-      <c r="B28" s="18" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>eye_of_ender</t>
         </is>
       </c>
-      <c r="C28" s="18" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Eye of Ender</t>
         </is>
@@ -1759,36 +1678,36 @@
           <t>Gain 1 Mulligan this round</t>
         </is>
       </c>
-      <c r="E28" s="18" t="n">
+      <c r="E28" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F28" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="18" t="n">
+      <c r="F28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="8" t="n">
         <v>20</v>
       </c>
-      <c r="H28" s="18" t="inlineStr">
+      <c r="H28" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I28" s="18" t="b">
+      <c r="I28" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>lucky_coin</t>
         </is>
       </c>
-      <c r="B29" s="18" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>lucky_coin</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>Lucky Coin</t>
         </is>
@@ -1798,36 +1717,36 @@
           <t>If you don't swap this hand, gain 1 extra swap next hand, If you do, gain +2 gold</t>
         </is>
       </c>
-      <c r="E29" s="18" t="n">
+      <c r="E29" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F29" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="18" t="n">
+      <c r="F29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="H29" s="18" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I29" s="18" t="b">
+      <c r="I29" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>holy_grail</t>
         </is>
       </c>
-      <c r="B30" s="18" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>holy_grail</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Holy Grail</t>
         </is>
@@ -1837,36 +1756,36 @@
           <t>Increase explosion limit by 1</t>
         </is>
       </c>
-      <c r="E30" s="18" t="n">
+      <c r="E30" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="18" t="n">
+      <c r="F30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="H30" s="18" t="inlineStr">
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I30" s="18" t="b">
+      <c r="I30" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>ice_cube</t>
         </is>
       </c>
-      <c r="B31" s="18" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>ice_cube</t>
         </is>
       </c>
-      <c r="C31" s="18" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Ice Cube</t>
         </is>
@@ -1876,36 +1795,36 @@
           <t>For the next 4 ingredients, explosiveness is added normally unless that ingredient would make the cauldron explode</t>
         </is>
       </c>
-      <c r="E31" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="18" t="n">
+      <c r="E31" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="8" t="n">
         <v>30</v>
       </c>
-      <c r="H31" s="18" t="inlineStr">
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I31" s="18" t="b">
+      <c r="I31" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>shrunken_head</t>
         </is>
       </c>
-      <c r="B32" s="18" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>shrunken_head</t>
         </is>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Shrunken Head</t>
         </is>
@@ -1915,36 +1834,36 @@
           <t>Your next hand is only 4 ingredients</t>
         </is>
       </c>
-      <c r="E32" s="18" t="n">
+      <c r="E32" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F32" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="18" t="n">
+      <c r="F32" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="8" t="n">
         <v>18</v>
       </c>
-      <c r="H32" s="18" t="inlineStr">
+      <c r="H32" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I32" s="18" t="b">
+      <c r="I32" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>jar_of_dirt</t>
         </is>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>jar_of_dirt</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Jar of Dirt</t>
         </is>
@@ -1954,36 +1873,36 @@
           <t>Add a pumpkin to your bag. Breaks after 5 pumpkins.</t>
         </is>
       </c>
-      <c r="E33" s="18" t="n">
+      <c r="E33" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F33" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="18" t="n">
+      <c r="F33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="H33" s="18" t="inlineStr">
+      <c r="H33" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I33" s="18" t="b">
+      <c r="I33" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="inlineStr">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>stirring_spoon</t>
         </is>
       </c>
-      <c r="B34" s="18" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>stirring_spoon</t>
         </is>
       </c>
-      <c r="C34" s="18" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>Stirring Spoon</t>
         </is>
@@ -1993,36 +1912,36 @@
           <t>Your next hand has an additional swap</t>
         </is>
       </c>
-      <c r="E34" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="18" t="n">
+      <c r="E34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="H34" s="18" t="inlineStr">
+      <c r="H34" s="8" t="inlineStr">
         <is>
           <t>uncommon</t>
         </is>
       </c>
-      <c r="I34" s="18" t="b">
+      <c r="I34" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>fish_bones</t>
         </is>
       </c>
-      <c r="B35" s="18" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>fish_bones</t>
         </is>
       </c>
-      <c r="C35" s="18" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Fish Bones</t>
         </is>
@@ -2032,36 +1951,36 @@
           <t>Reduce your cauldron's score by 1 and gain 2 gold</t>
         </is>
       </c>
-      <c r="E35" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="18" t="n">
+      <c r="E35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H35" s="18" t="inlineStr">
+      <c r="H35" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I35" s="18" t="b">
+      <c r="I35" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="inlineStr">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>fairy_in_a_cage</t>
         </is>
       </c>
-      <c r="B36" s="18" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>fairy_in_a_cage</t>
         </is>
       </c>
-      <c r="C36" s="18" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Fairy in a Cage</t>
         </is>
@@ -2071,36 +1990,36 @@
           <t>Your next ingredient disappears forever</t>
         </is>
       </c>
-      <c r="E36" s="18" t="n">
+      <c r="E36" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F36" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="18" t="n">
+      <c r="F36" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="H36" s="18" t="inlineStr">
+      <c r="H36" s="8" t="inlineStr">
         <is>
           <t>legendary</t>
         </is>
       </c>
-      <c r="I36" s="18" t="b">
+      <c r="I36" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>booberry</t>
         </is>
       </c>
-      <c r="B37" s="18" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>booberry</t>
         </is>
       </c>
-      <c r="C37" s="18" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Boo-berry</t>
         </is>
@@ -2110,36 +2029,36 @@
           <t>End of hand: lose 2 explosiveness</t>
         </is>
       </c>
-      <c r="E37" s="18" t="n">
+      <c r="E37" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F37" s="18" t="n">
+      <c r="F37" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="18" t="n">
+      <c r="G37" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="H37" s="18" t="inlineStr">
+      <c r="H37" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I37" s="18" t="b">
+      <c r="I37" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>chicken</t>
         </is>
       </c>
-      <c r="B38" s="18" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>chicken</t>
         </is>
       </c>
-      <c r="C38" s="18" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>Chicken</t>
         </is>
@@ -2149,36 +2068,36 @@
           <t>This cannot make your cauldron explode</t>
         </is>
       </c>
-      <c r="E38" s="18" t="n">
+      <c r="E38" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F38" s="18" t="n">
+      <c r="F38" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="G38" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="18" t="inlineStr">
+      <c r="G38" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I38" s="18" t="b">
+      <c r="I38" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="inlineStr">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>spider</t>
         </is>
       </c>
-      <c r="B39" s="18" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>spider</t>
         </is>
       </c>
-      <c r="C39" s="18" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>Spider</t>
         </is>
@@ -2188,36 +2107,36 @@
           <t>TBD</t>
         </is>
       </c>
-      <c r="E39" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="18" t="n">
+      <c r="E39" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="H39" s="18" t="inlineStr">
+      <c r="H39" s="8" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="I39" s="18" t="b">
+      <c r="I39" s="8" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>poison_apple</t>
         </is>
       </c>
-      <c r="B40" s="18" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>poison_apple</t>
         </is>
       </c>
-      <c r="C40" s="18" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>Poison Apple</t>
         </is>
@@ -2227,36 +2146,36 @@
           <t>In 2 hands, gain 3 explosiveness</t>
         </is>
       </c>
-      <c r="E40" s="18" t="n">
+      <c r="E40" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F40" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="18" t="n">
+      <c r="F40" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="H40" s="18" t="inlineStr">
+      <c r="H40" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I40" s="18" t="b">
+      <c r="I40" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="18" t="inlineStr">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>cobbler</t>
         </is>
       </c>
-      <c r="B41" s="18" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>cobbler</t>
         </is>
       </c>
-      <c r="C41" s="18" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>Cobbler</t>
         </is>
@@ -2266,36 +2185,36 @@
           <t>Adjacent Boomberries are +2 explosiveness and +10 score</t>
         </is>
       </c>
-      <c r="E41" s="18" t="n">
+      <c r="E41" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="18" t="n">
+      <c r="F41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="H41" s="18" t="inlineStr">
+      <c r="H41" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I41" s="18" t="b">
+      <c r="I41" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="18" t="inlineStr">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>growth_potion</t>
         </is>
       </c>
-      <c r="B42" s="18" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>growth_potion</t>
         </is>
       </c>
-      <c r="C42" s="18" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t>Growth Potion</t>
         </is>
@@ -2305,36 +2224,36 @@
           <t>The next 4 ingredients stats are doubled</t>
         </is>
       </c>
-      <c r="E42" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="18" t="n">
+      <c r="E42" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="8" t="n">
         <v>40</v>
       </c>
-      <c r="H42" s="18" t="inlineStr">
+      <c r="H42" s="8" t="inlineStr">
         <is>
           <t>epic</t>
         </is>
       </c>
-      <c r="I42" s="18" t="b">
+      <c r="I42" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="inlineStr">
+      <c r="A43" s="8" t="inlineStr">
         <is>
           <t>severed_right_hand</t>
         </is>
       </c>
-      <c r="B43" s="18" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t>severed_right_hand</t>
         </is>
       </c>
-      <c r="C43" s="18" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
         <is>
           <t>Severed Right Hand</t>
         </is>
@@ -2344,36 +2263,36 @@
           <t>Gains 1 score for each ingredient to the left</t>
         </is>
       </c>
-      <c r="E43" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" s="18" t="n">
+      <c r="E43" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="H43" s="18" t="inlineStr">
+      <c r="H43" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I43" s="18" t="b">
+      <c r="I43" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="18" t="inlineStr">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>severed_left_hand</t>
         </is>
       </c>
-      <c r="B44" s="18" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>severed_left_hand</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
         <is>
           <t>Severed Left Hand</t>
         </is>
@@ -2383,36 +2302,36 @@
           <t>Gains 1 score for each ingredient to the right</t>
         </is>
       </c>
-      <c r="E44" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" s="18" t="n">
+      <c r="E44" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="H44" s="18" t="inlineStr">
+      <c r="H44" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I44" s="18" t="b">
+      <c r="I44" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="18" t="inlineStr">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>juggling_club</t>
         </is>
       </c>
-      <c r="B45" s="18" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t>juggling_club</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
         <is>
           <t>Juggling Club</t>
         </is>
@@ -2422,36 +2341,36 @@
           <t>Your next 3 hands have an additional swap</t>
         </is>
       </c>
-      <c r="E45" s="18" t="n">
+      <c r="E45" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="F45" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" s="18" t="n">
+      <c r="F45" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="H45" s="18" t="inlineStr">
+      <c r="H45" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I45" s="18" t="b">
+      <c r="I45" s="8" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="18" t="inlineStr">
+      <c r="A46" s="8" t="inlineStr">
         <is>
           <t>honey</t>
         </is>
       </c>
-      <c r="B46" s="18" t="inlineStr">
+      <c r="B46" s="8" t="inlineStr">
         <is>
           <t>honey</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C46" s="8" t="inlineStr">
         <is>
           <t>Honey</t>
         </is>
@@ -2461,21 +2380,21 @@
           <t>The ingredient to the left</t>
         </is>
       </c>
-      <c r="E46" s="18" t="n">
+      <c r="E46" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F46" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="18" t="n">
+      <c r="F46" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="H46" s="18" t="inlineStr">
+      <c r="H46" s="8" t="inlineStr">
         <is>
           <t>rare</t>
         </is>
       </c>
-      <c r="I46" s="18" t="b">
+      <c r="I46" s="8" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2506,64 +2425,64 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>ingredient_id</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>boom_berry_1</t>
         </is>
       </c>
-      <c r="B2" s="18" t="n">
+      <c r="B2" s="8" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>pumpkin</t>
         </is>
       </c>
-      <c r="B3" s="18" t="n">
+      <c r="B3" s="8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>rat</t>
         </is>
       </c>
-      <c r="B4" s="18" t="n">
+      <c r="B4" s="8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>red_mushroom</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="8" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>boom_berry_2</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="8" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2592,452 +2511,452 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="D1" s="17" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>pool</t>
         </is>
       </c>
-      <c r="E1" s="17" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>pool_unlock_level</t>
         </is>
       </c>
-      <c r="F1" s="17" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>explosion_limit_modifier</t>
         </is>
       </c>
-      <c r="G1" s="17" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>score_multiplier_percent</t>
         </is>
       </c>
-      <c r="H1" s="17" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>gold_multiplier_percent</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>stable_brew</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Stable Brew</t>
         </is>
       </c>
-      <c r="C2" s="18" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Explosion limit +1 this level.</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E2" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="18" t="n">
+      <c r="E2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H2" s="18" t="n">
+      <c r="H2" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>gold_rush</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Gold Rush</t>
         </is>
       </c>
-      <c r="C3" s="18" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>Gold earned +25% this level.</t>
         </is>
       </c>
-      <c r="D3" s="18" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E3" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="18" t="n">
+      <c r="E3" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H3" s="18" t="n">
+      <c r="H3" s="8" t="n">
         <v>125</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>shaky_hands</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Shaky Hands</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Explosion limit -1 this level.</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E4" s="18" t="n">
+      <c r="E4" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="8" t="n">
         <v>-1</v>
       </c>
-      <c r="G4" s="18" t="n">
+      <c r="G4" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H4" s="18" t="n">
+      <c r="H4" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>volatile_brew</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Volatile Brew</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Explosion limit -2.</t>
         </is>
       </c>
-      <c r="D5" s="18" t="inlineStr">
+      <c r="D5" s="8" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="8" t="n">
         <v>-2</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>stingy</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Stingy</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Gold earned -25%.</t>
         </is>
       </c>
-      <c r="D6" s="18" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E6" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="18" t="n">
+      <c r="E6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="8" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>low_expectations</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Low Expectations</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Threshold reduced by 15%</t>
         </is>
       </c>
-      <c r="D7" s="18" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E7" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="18" t="n">
+      <c r="E7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8" t="n">
         <v>85</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>under_pressure</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Under Pressure</t>
         </is>
       </c>
-      <c r="C8" s="18" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>Increase threshold and gold gain by 15%</t>
         </is>
       </c>
-      <c r="D8" s="18" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E8" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="18" t="n">
+      <c r="E8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="8" t="n">
         <v>115</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="8" t="n">
         <v>115</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>in_rhythm</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>In Rhythm</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>every 3rd ingredient added to the cauldron has double score and explosiveness</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E9" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="18" t="n">
+      <c r="E9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="H9" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>practice brew</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Practice Brew</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>You may restart the brew at anypoint before it explodes</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E10" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="18" t="n">
+      <c r="E10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>regular_brew</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Regular Brew</t>
         </is>
       </c>
-      <c r="C11" s="18" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Nothing special</t>
         </is>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="18" t="n">
+      <c r="E11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="H11" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>regular_boss</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Regular Boss</t>
         </is>
       </c>
-      <c r="C12" s="18" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Nothing special</t>
         </is>
       </c>
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="8" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="18" t="n">
+      <c r="E12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="H12" s="8" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>bubbling_brew</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Bubbling Brew</t>
         </is>
       </c>
-      <c r="C13" s="18" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>every 3rd ingredient added to the cauldron jumps back into your bag.</t>
         </is>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="18" t="n">
+      <c r="E13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="8" t="n">
         <v>100</v>
       </c>
     </row>
@@ -3066,29 +2985,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="17" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>display_name</t>
         </is>
       </c>
-      <c r="C1" s="17" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>pumpkin_trinket</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Pumpkin Necklace</t>
         </is>
@@ -3100,12 +3019,12 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>red_mushroom_trinket</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Red Mushroom Trinket</t>
         </is>
@@ -3117,12 +3036,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>rat_trinket</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Rat Trinket</t>
         </is>
@@ -3134,12 +3053,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>jar_of_flies</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Jar of Flies</t>
         </is>
@@ -3151,12 +3070,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>pocket_watch</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Pocket Watch</t>
         </is>
@@ -3168,12 +3087,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>time_turner</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Time Turner</t>
         </is>
@@ -3185,12 +3104,12 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>jar_of_froglegs</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Jar of Froglegs</t>
         </is>
@@ -3202,12 +3121,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>voodoo_doll_trinket</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Voodoo Doll</t>
         </is>
@@ -3219,12 +3138,12 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>pristine_feather</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Pristine Feather</t>
         </is>
@@ -3236,12 +3155,12 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>beating_heart</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Beating Heart</t>
         </is>
@@ -3253,12 +3172,12 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>gecko_feet</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Gecko Feet</t>
         </is>

</xml_diff>

<commit_message>
Implement Gecko Assistant, Bubbling Brew, and brew UX fixes
- Add gecko_assistant trinket: every 9th hand play stays in hand with countdown UI and art
- Implement Bubbling Brew aura: every 3rd ingredient returns to bag with fly animation and previews
- Fix Cobbler/Boom Berry crash on boss clear when prior hand slot is empty
- Smaller in-brew mulligan purchase icon; hide buy option when gold is insufficient
- Sync trinket data and spreadsheet; add Beating Heart and Gecko Assistant art
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -3174,17 +3174,17 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>gecko_feet</t>
+          <t>gecko_assistant</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Gecko Feet</t>
+          <t>Gecko Assistant</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Every 11 ingredients stays in your hand</t>
+          <t>Every 9th ingredient stays in your hand</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Headless Chicken trinket and unified hand preview resolution
- Headless Chicken: block chicken draws for first 2 hand draws per brew, with trinket countdown

- Unified HandPlayPreview for stats, shakes, and effect icons (honey, gecko, bat wing, parrot, etc.)

- Fix hand row visibility during incremental draw animations

- Export spreadsheet updates for trinkets, ingredients, and auras
</commit_message>
<xml_diff>
--- a/data/ingredients.xlsx
+++ b/data/ingredients.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\Alchemy Roguelite Godot\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F21427A-2EE9-45B6-AC24-D220C46FBB24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD281E10-D8D0-4798-A2A8-735BD7ECDDD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="239">
   <si>
     <t>id</t>
   </si>
@@ -732,6 +732,15 @@
   </si>
   <si>
     <t>Does not play the ingredient to the left</t>
+  </si>
+  <si>
+    <t>headless_chicken</t>
+  </si>
+  <si>
+    <t>Headless Chicken</t>
+  </si>
+  <si>
+    <t>You cannot draw chickens for the first 2 turns</t>
   </si>
 </sst>
 </file>
@@ -2971,7 +2980,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -3111,6 +3120,17 @@
         <v>35</v>
       </c>
     </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C13" t="s">
+        <v>238</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>